<commit_message>
Research workbook: ask title companies about off-market share
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D3BAjidWEHgnEjgiFZcuRg
</commit_message>
<xml_diff>
--- a/research-template.xlsx
+++ b/research-template.xlsx
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="350">
   <si>
     <t xml:space="preserve">Market Research Workbook</t>
   </si>
@@ -510,6 +510,9 @@
   </si>
   <si>
     <t xml:space="preserve">•  Who are the active flippers? Which lenders and contractors do they use?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Title companies: what share of your closings are off-market or wholesale deals?</t>
   </si>
   <si>
     <t xml:space="preserve">•  Would you work with an out-of-state buyer? What do you need from me?</t>
@@ -2094,7 +2097,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:D49"/>
+  <dimension ref="B1:D50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -2442,17 +2445,17 @@
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="3" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="14" t="s">
+      <c r="B47" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="14" t="s">
@@ -2468,8 +2471,15 @@
       <c r="C49" s="14"/>
       <c r="D49" s="14"/>
     </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C14:D14"/>
@@ -2487,9 +2497,10 @@
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B43:D43"/>
     <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B45:D45"/>
     <mergeCell ref="B48:D48"/>
     <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B50:D50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C24" r:id="rId1" display="Redfin ZIP housing market page&#10;https://www.redfin.com/zipcode/44102/housing-market"/>
@@ -2538,17 +2549,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D3" s="58" t="n">
         <f aca="false">COUNTA(C8:C307)</f>
@@ -2557,19 +2568,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D4" s="59" t="n">
         <f aca="false">IFERROR(AVERAGE(O8:O307),"")</f>
         <v>0.0330188679245284</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D5" s="57" t="str">
         <f aca="false">IF(COUNT(O8:O307)=0,"",COUNTIF(O8:O307,"&lt;=0.1")&amp;" of "&amp;COUNT(O8:O307))</f>
@@ -2578,24 +2589,24 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
       <c r="E6" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F6" s="17"/>
       <c r="G6" s="17"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="M6" s="17"/>
       <c r="N6" s="17"/>
@@ -2603,49 +2614,49 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2653,10 +2664,10 @@
         <v>46300</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D8" s="36" t="n">
         <v>1200</v>
@@ -2680,7 +2691,7 @@
         <v>212000</v>
       </c>
       <c r="K8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L8" s="48" t="str">
         <f aca="false">IF(OR(F8="",I8=""),"",IF(F8&gt;=I8,"Yes","No"))</f>
@@ -11417,30 +11428,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="X5" s="16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AH5" s="9" t="n">
         <f aca="false">SUM(X6:AG6)</f>
         <v>100</v>
       </c>
       <c r="AI5" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17"/>
       <c r="B6" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
@@ -11449,31 +11460,31 @@
       <c r="G6" s="17"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M6" s="17"/>
       <c r="N6" s="17"/>
       <c r="O6" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P6" s="17"/>
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
       <c r="S6" s="17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="T6" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U6" s="17"/>
       <c r="V6" s="17"/>
       <c r="W6" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="X6" s="18" t="n">
         <v>15</v>
@@ -11508,108 +11519,108 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="S7" s="19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="T7" s="19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="U7" s="19" t="s">
         <v>57</v>
       </c>
       <c r="V7" s="19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X7" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Y7" s="19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Z7" s="19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AA7" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AB7" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AC7" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AD7" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AE7" s="19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AF7" s="19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG7" s="19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="21" t="n">
         <f aca="false">IF($A8="","",COUNTIF(ZIPs!$A$8:$A$107,$A8))</f>
@@ -12347,36 +12358,36 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I17" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12555,7 +12566,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -12638,22 +12649,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
@@ -12662,20 +12673,20 @@
       <c r="I6" s="17"/>
       <c r="J6" s="17"/>
       <c r="K6" s="17" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="M6" s="17"/>
       <c r="N6" s="17"/>
       <c r="O6" s="17"/>
       <c r="P6" s="17" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Q6" s="17"/>
       <c r="R6" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S6" s="17"/>
       <c r="T6" s="17"/>
@@ -12683,100 +12694,100 @@
       <c r="V6" s="17"/>
       <c r="W6" s="17"/>
       <c r="X6" s="17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Y6" s="17"/>
       <c r="Z6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L7" s="19" t="s">
         <v>48</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="S7" s="19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T7" s="19" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="U7" s="19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V7" s="19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="X7" s="19" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Y7" s="19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Z7" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D8" s="35" t="n">
         <v>185000</v>
@@ -12818,7 +12829,7 @@
         <v>46310</v>
       </c>
       <c r="Q8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R8" s="39" t="n">
         <f aca="false">IF(OR(E8="",F8="",E8=0),"",F8/(E8/3))</f>
@@ -18346,17 +18357,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -18366,7 +18377,7 @@
       <c r="G6" s="17"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
@@ -18377,7 +18388,7 @@
       <c r="P6" s="17"/>
       <c r="Q6" s="17"/>
       <c r="R6" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S6" s="17"/>
       <c r="T6" s="17"/>
@@ -18386,81 +18397,81 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="S7" s="19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="T7" s="19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="U7" s="19" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="V7" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D8" s="30"/>
       <c r="E8" s="36" t="n">
@@ -18473,7 +18484,7 @@
         <v>1150</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I8" s="38" t="n">
         <v>46266</v>
@@ -18485,7 +18496,7 @@
         <v>139900</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M8" s="38" t="n">
         <v>46297</v>
@@ -18496,7 +18507,7 @@
         <v>46310</v>
       </c>
       <c r="Q8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R8" s="24" t="n">
         <f aca="false">IF(OR(J8="",K8="",J8=0),"",1-K8/J8)</f>
@@ -30234,17 +30245,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -30255,12 +30266,12 @@
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
       <c r="J6" s="17" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="N6" s="17"/>
       <c r="O6" s="17"/>
@@ -30270,69 +30281,69 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D8" s="30"/>
       <c r="E8" s="36" t="n">
@@ -30357,7 +30368,7 @@
         <v>112000</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M8" s="46" t="n">
         <f aca="false">IF(OR(H8="",E8="",E8=0),"",H8/E8)</f>
@@ -37990,45 +38001,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E3" s="49" t="n">
         <v>30</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E4" s="50" t="n">
         <v>0.1</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
       <c r="E6" s="17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F6" s="17"/>
       <c r="G6" s="17"/>
@@ -38038,7 +38049,7 @@
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
       <c r="M6" s="17" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N6" s="17"/>
       <c r="O6" s="17"/>
@@ -38050,75 +38061,75 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="R7" s="19" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="S7" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="T7" s="19" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D8" s="36" t="n">
         <v>1300</v>
@@ -38137,13 +38148,13 @@
       </c>
       <c r="I8" s="41"/>
       <c r="J8" s="20" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K8" s="20" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M8" s="39" t="n">
         <f aca="false">IF(OR(E8="",G8=""),"",(G8-E8)/30.44)</f>
@@ -51967,52 +51978,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -53650,17 +53661,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -53668,14 +53679,14 @@
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
       <c r="G6" s="17" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
       <c r="L6" s="17" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="M6" s="17"/>
       <c r="N6" s="17"/>
@@ -53684,72 +53695,72 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O7" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" s="38" t="n">
         <v>46307</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G8" s="35" t="n">
         <v>215000</v>
@@ -53767,19 +53778,19 @@
         <v>3</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="M8" s="20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="N8" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P8" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -59213,38 +59224,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B7" s="27" t="n">
         <v>1200</v>
@@ -59252,7 +59263,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B8" s="41" t="n">
         <v>135000</v>
@@ -59260,32 +59271,32 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B11" s="51" t="s">
+        <v>187</v>
+      </c>
+      <c r="C11" s="51" t="s">
+        <v>179</v>
+      </c>
+      <c r="D11" s="51" t="s">
         <v>186</v>
       </c>
-      <c r="C11" s="51" t="s">
-        <v>178</v>
-      </c>
-      <c r="D11" s="51" t="s">
-        <v>185</v>
-      </c>
       <c r="E11" s="51" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F11" s="51" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B12" s="41" t="n">
         <v>212000</v>
@@ -59306,7 +59317,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B13" s="41" t="n">
         <v>205000</v>
@@ -59327,7 +59338,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B14" s="41" t="n">
         <v>219500</v>
@@ -59370,7 +59381,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B18" s="46" t="n">
         <f aca="false">IFERROR(MIN(F12:F16),"")</f>
@@ -59379,7 +59390,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B19" s="46" t="n">
         <f aca="false">IFERROR(MEDIAN(F12:F16),"")</f>
@@ -59388,7 +59399,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B20" s="52" t="n">
         <f aca="false">IF(OR(B18="",B18=0,B7=""),"",B18*B7)</f>
@@ -59397,7 +59408,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B21" s="46" t="n">
         <f aca="false">IF(OR(B19="",B19=0,B7=""),"",B19*B7)</f>
@@ -59406,18 +59417,18 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B24" s="41"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B25" s="52" t="n">
         <f aca="false">IF(B24&lt;&gt;"",B24,B20)</f>
@@ -59426,7 +59437,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B26" s="41" t="n">
         <v>120000</v>
@@ -59434,7 +59445,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B27" s="31" t="n">
         <v>0.02</v>
@@ -59442,7 +59453,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B28" s="41" t="n">
         <v>35000</v>
@@ -59450,7 +59461,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B29" s="31" t="n">
         <v>0.2</v>
@@ -59458,7 +59469,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B30" s="27" t="n">
         <v>6</v>
@@ -59466,7 +59477,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B31" s="41" t="n">
         <v>650</v>
@@ -59474,7 +59485,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B32" s="31" t="n">
         <v>0.08</v>
@@ -59482,7 +59493,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B33" s="31" t="n">
         <v>0</v>
@@ -59490,7 +59501,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B34" s="31" t="n">
         <v>0.11</v>
@@ -59498,7 +59509,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B35" s="31" t="n">
         <v>0.02</v>
@@ -59506,7 +59517,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B36" s="31" t="n">
         <v>0.15</v>
@@ -59514,12 +59525,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B39" s="46" t="n">
         <f aca="false">B26*B27</f>
@@ -59528,7 +59539,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B40" s="46" t="n">
         <f aca="false">B28*(1+B29)</f>
@@ -59537,7 +59548,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B41" s="46" t="n">
         <f aca="false">B30*B31</f>
@@ -59546,7 +59557,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B42" s="46" t="n">
         <f aca="false">B33*(B26+B40)</f>
@@ -59555,7 +59566,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B43" s="46" t="n">
         <f aca="false">B42*B34*B30/12+B42*B35</f>
@@ -59564,7 +59575,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B44" s="46" t="n">
         <f aca="false">IF(B25="","",B25*B32)</f>
@@ -59573,7 +59584,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B45" s="46" t="n">
         <f aca="false">IF(B25="","",B26+B39+B40+B41+B43+B44)</f>
@@ -59582,7 +59593,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B46" s="52" t="n">
         <f aca="false">IF(B25="","",B25-B45)</f>
@@ -59591,7 +59602,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B47" s="46" t="n">
         <f aca="false">B26+B39+B40+B41+B43-B42</f>
@@ -59600,7 +59611,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="9" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B48" s="53" t="n">
         <f aca="false">IF(OR(B46="",B25=0),"",B46/B25)</f>
@@ -59609,7 +59620,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B49" s="53" t="n">
         <f aca="false">IF(OR(B46="",B47&lt;=0),"",B46/B47)</f>
@@ -59618,56 +59629,56 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B50" s="52" t="n">
         <f aca="false">IF(B25="","",(B25*(1-B32-B36)-B40-B41-B33*B40*(B34*B30/12+B35))/(1+B27+B33*(B34*B30/12+B35)))</f>
         <v>105637.254901961</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B51" s="46" t="n">
         <f aca="false">IF(B25="","",B25*0.7-B40)</f>
         <v>97681.8181818182</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="54" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B54" s="54" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C54" s="54" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D54" s="54" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E54" s="54" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F54" s="54" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="55" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B55" s="46" t="n">
         <f aca="false">IF($B$25="","",B25)</f>
@@ -59692,7 +59703,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="55" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B56" s="46" t="n">
         <f aca="false">IF($B$25="","",B25*0.9)</f>
@@ -59717,7 +59728,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="55" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B57" s="46" t="n">
         <f aca="false">IF($B$25="","",B25)</f>
@@ -59742,7 +59753,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="55" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B58" s="46" t="n">
         <f aca="false">IF($B$25="","",B25)</f>
@@ -59767,7 +59778,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="56" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B59" s="46" t="n">
         <f aca="false">IF($B$25="","",B25*0.9)</f>
@@ -59792,7 +59803,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B61" s="57" t="str">
         <f aca="false">IF(E59="","",IF(E59&gt;0,"YES: still profitable","NO: too thin"))</f>
@@ -59803,12 +59814,12 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B64" s="30"/>
       <c r="C64" s="30"/>
@@ -59816,25 +59827,25 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B65" s="30"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B66" s="30"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B67" s="30"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B68" s="30"/>
     </row>

</xml_diff>

<commit_message>
Research pack: drop un-starred metros from the workbook; room for 10 metros
Update my workbook now clears rows OfferDesk filled for metros that are no
longer starred (rows he typed in are kept and named in the message). The
Metros tab holds 10 metros; older workbooks are moved into the new template
on update, keeping everything he typed (Ready check answers move with their
metro).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D3BAjidWEHgnEjgiFZcuRg
</commit_message>
<xml_diff>
--- a/research-template.xlsx
+++ b/research-template.xlsx
@@ -11404,7 +11404,7 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AI25"/>
+  <dimension ref="A1:AI33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -11706,43 +11706,43 @@
         <v>100</v>
       </c>
       <c r="X8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",D8=""),"",IF(COUNT(D$8:D$13)&lt;2,1,(COUNT(D$8:D$13)-RANK(D8,D$8:D$13,0))/(COUNT(D$8:D$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",D8=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D8,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="Y8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",E8=""),"",IF(COUNT(E$8:E$13)&lt;2,1,(COUNT(E$8:E$13)-RANK(E8,E$8:E$13,1))/(COUNT(E$8:E$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",E8=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E8,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="Z8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",F8=""),"",IF(COUNT(F$8:F$13)&lt;2,1,(COUNT(F$8:F$13)-RANK(F8,F$8:F$13,0))/(COUNT(F$8:F$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",F8=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F8,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AA8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",G8=""),"",IF(COUNT(G$8:G$13)&lt;2,1,(COUNT(G$8:G$13)-RANK(G8,G$8:G$13,0))/(COUNT(G$8:G$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",G8=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G8,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AB8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",J8=""),"",IF(COUNT(J$8:J$13)&lt;2,1,(COUNT(J$8:J$13)-RANK(J8,J$8:J$13,1))/(COUNT(J$8:J$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",J8=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J8,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AC8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",P8=""),"",IF(COUNT(P$8:P$13)&lt;2,1,(COUNT(P$8:P$13)-RANK(P8,P$8:P$13,1))/(COUNT(P$8:P$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",P8=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P8,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AD8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",S8=""),"",IF(COUNT(S$8:S$13)&lt;2,1,(COUNT(S$8:S$13)-RANK(S8,S$8:S$13,1))/(COUNT(S$8:S$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",S8=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S8,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AE8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",T8=""),"",IF(COUNT(T$8:T$13)&lt;2,1,(COUNT(T$8:T$13)-RANK(T8,T$8:T$13,0))/(COUNT(T$8:T$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",T8=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T8,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AF8" s="29" t="n">
-        <f aca="false">IF(OR($A8="",U8=""),"",IF(COUNT(U$8:U$13)&lt;2,1,(COUNT(U$8:U$13)-RANK(U8,U$8:U$13,0))/(COUNT(U$8:U$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",U8=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U8,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
         <v>1</v>
       </c>
       <c r="AG8" s="29" t="str">
-        <f aca="false">IF(OR($A8="",V8=""),"",IF(COUNT(V$8:V$13)&lt;2,1,(COUNT(V$8:V$13)-RANK(V8,V$8:V$13,0))/(COUNT(V$8:V$13)-1)))</f>
+        <f aca="false">IF(OR($A8="",V8=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V8,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
         <v/>
       </c>
     </row>
@@ -11828,43 +11828,43 @@
         <v/>
       </c>
       <c r="X9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",D9=""),"",IF(COUNT(D$8:D$13)&lt;2,1,(COUNT(D$8:D$13)-RANK(D9,D$8:D$13,0))/(COUNT(D$8:D$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",D9=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D9,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
         <v/>
       </c>
       <c r="Y9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",E9=""),"",IF(COUNT(E$8:E$13)&lt;2,1,(COUNT(E$8:E$13)-RANK(E9,E$8:E$13,1))/(COUNT(E$8:E$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",E9=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E9,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
         <v/>
       </c>
       <c r="Z9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",F9=""),"",IF(COUNT(F$8:F$13)&lt;2,1,(COUNT(F$8:F$13)-RANK(F9,F$8:F$13,0))/(COUNT(F$8:F$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",F9=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F9,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
         <v/>
       </c>
       <c r="AA9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",G9=""),"",IF(COUNT(G$8:G$13)&lt;2,1,(COUNT(G$8:G$13)-RANK(G9,G$8:G$13,0))/(COUNT(G$8:G$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",G9=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G9,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
         <v/>
       </c>
       <c r="AB9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",J9=""),"",IF(COUNT(J$8:J$13)&lt;2,1,(COUNT(J$8:J$13)-RANK(J9,J$8:J$13,1))/(COUNT(J$8:J$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",J9=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J9,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
         <v/>
       </c>
       <c r="AC9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",P9=""),"",IF(COUNT(P$8:P$13)&lt;2,1,(COUNT(P$8:P$13)-RANK(P9,P$8:P$13,1))/(COUNT(P$8:P$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",P9=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P9,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
         <v/>
       </c>
       <c r="AD9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",S9=""),"",IF(COUNT(S$8:S$13)&lt;2,1,(COUNT(S$8:S$13)-RANK(S9,S$8:S$13,1))/(COUNT(S$8:S$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",S9=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S9,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
         <v/>
       </c>
       <c r="AE9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",T9=""),"",IF(COUNT(T$8:T$13)&lt;2,1,(COUNT(T$8:T$13)-RANK(T9,T$8:T$13,0))/(COUNT(T$8:T$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",T9=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T9,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
         <v/>
       </c>
       <c r="AF9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",U9=""),"",IF(COUNT(U$8:U$13)&lt;2,1,(COUNT(U$8:U$13)-RANK(U9,U$8:U$13,0))/(COUNT(U$8:U$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",U9=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U9,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
         <v/>
       </c>
       <c r="AG9" s="29" t="str">
-        <f aca="false">IF(OR($A9="",V9=""),"",IF(COUNT(V$8:V$13)&lt;2,1,(COUNT(V$8:V$13)-RANK(V9,V$8:V$13,0))/(COUNT(V$8:V$13)-1)))</f>
+        <f aca="false">IF(OR($A9="",V9=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V9,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
         <v/>
       </c>
     </row>
@@ -11950,43 +11950,43 @@
         <v/>
       </c>
       <c r="X10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",D10=""),"",IF(COUNT(D$8:D$13)&lt;2,1,(COUNT(D$8:D$13)-RANK(D10,D$8:D$13,0))/(COUNT(D$8:D$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",D10=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D10,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
         <v/>
       </c>
       <c r="Y10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",E10=""),"",IF(COUNT(E$8:E$13)&lt;2,1,(COUNT(E$8:E$13)-RANK(E10,E$8:E$13,1))/(COUNT(E$8:E$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",E10=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E10,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
         <v/>
       </c>
       <c r="Z10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",F10=""),"",IF(COUNT(F$8:F$13)&lt;2,1,(COUNT(F$8:F$13)-RANK(F10,F$8:F$13,0))/(COUNT(F$8:F$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",F10=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F10,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
         <v/>
       </c>
       <c r="AA10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",G10=""),"",IF(COUNT(G$8:G$13)&lt;2,1,(COUNT(G$8:G$13)-RANK(G10,G$8:G$13,0))/(COUNT(G$8:G$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",G10=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G10,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
         <v/>
       </c>
       <c r="AB10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",J10=""),"",IF(COUNT(J$8:J$13)&lt;2,1,(COUNT(J$8:J$13)-RANK(J10,J$8:J$13,1))/(COUNT(J$8:J$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",J10=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J10,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
         <v/>
       </c>
       <c r="AC10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",P10=""),"",IF(COUNT(P$8:P$13)&lt;2,1,(COUNT(P$8:P$13)-RANK(P10,P$8:P$13,1))/(COUNT(P$8:P$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",P10=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P10,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
         <v/>
       </c>
       <c r="AD10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",S10=""),"",IF(COUNT(S$8:S$13)&lt;2,1,(COUNT(S$8:S$13)-RANK(S10,S$8:S$13,1))/(COUNT(S$8:S$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",S10=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S10,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
         <v/>
       </c>
       <c r="AE10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",T10=""),"",IF(COUNT(T$8:T$13)&lt;2,1,(COUNT(T$8:T$13)-RANK(T10,T$8:T$13,0))/(COUNT(T$8:T$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",T10=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T10,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
         <v/>
       </c>
       <c r="AF10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",U10=""),"",IF(COUNT(U$8:U$13)&lt;2,1,(COUNT(U$8:U$13)-RANK(U10,U$8:U$13,0))/(COUNT(U$8:U$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",U10=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U10,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
         <v/>
       </c>
       <c r="AG10" s="29" t="str">
-        <f aca="false">IF(OR($A10="",V10=""),"",IF(COUNT(V$8:V$13)&lt;2,1,(COUNT(V$8:V$13)-RANK(V10,V$8:V$13,0))/(COUNT(V$8:V$13)-1)))</f>
+        <f aca="false">IF(OR($A10="",V10=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V10,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
         <v/>
       </c>
     </row>
@@ -12072,43 +12072,43 @@
         <v/>
       </c>
       <c r="X11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",D11=""),"",IF(COUNT(D$8:D$13)&lt;2,1,(COUNT(D$8:D$13)-RANK(D11,D$8:D$13,0))/(COUNT(D$8:D$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",D11=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D11,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
         <v/>
       </c>
       <c r="Y11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",E11=""),"",IF(COUNT(E$8:E$13)&lt;2,1,(COUNT(E$8:E$13)-RANK(E11,E$8:E$13,1))/(COUNT(E$8:E$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",E11=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E11,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
         <v/>
       </c>
       <c r="Z11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",F11=""),"",IF(COUNT(F$8:F$13)&lt;2,1,(COUNT(F$8:F$13)-RANK(F11,F$8:F$13,0))/(COUNT(F$8:F$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",F11=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F11,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
         <v/>
       </c>
       <c r="AA11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",G11=""),"",IF(COUNT(G$8:G$13)&lt;2,1,(COUNT(G$8:G$13)-RANK(G11,G$8:G$13,0))/(COUNT(G$8:G$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",G11=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G11,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
         <v/>
       </c>
       <c r="AB11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",J11=""),"",IF(COUNT(J$8:J$13)&lt;2,1,(COUNT(J$8:J$13)-RANK(J11,J$8:J$13,1))/(COUNT(J$8:J$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",J11=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J11,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
         <v/>
       </c>
       <c r="AC11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",P11=""),"",IF(COUNT(P$8:P$13)&lt;2,1,(COUNT(P$8:P$13)-RANK(P11,P$8:P$13,1))/(COUNT(P$8:P$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",P11=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P11,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
         <v/>
       </c>
       <c r="AD11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",S11=""),"",IF(COUNT(S$8:S$13)&lt;2,1,(COUNT(S$8:S$13)-RANK(S11,S$8:S$13,1))/(COUNT(S$8:S$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",S11=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S11,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
         <v/>
       </c>
       <c r="AE11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",T11=""),"",IF(COUNT(T$8:T$13)&lt;2,1,(COUNT(T$8:T$13)-RANK(T11,T$8:T$13,0))/(COUNT(T$8:T$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",T11=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T11,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
         <v/>
       </c>
       <c r="AF11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",U11=""),"",IF(COUNT(U$8:U$13)&lt;2,1,(COUNT(U$8:U$13)-RANK(U11,U$8:U$13,0))/(COUNT(U$8:U$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",U11=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U11,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
         <v/>
       </c>
       <c r="AG11" s="29" t="str">
-        <f aca="false">IF(OR($A11="",V11=""),"",IF(COUNT(V$8:V$13)&lt;2,1,(COUNT(V$8:V$13)-RANK(V11,V$8:V$13,0))/(COUNT(V$8:V$13)-1)))</f>
+        <f aca="false">IF(OR($A11="",V11=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V11,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
         <v/>
       </c>
     </row>
@@ -12194,43 +12194,43 @@
         <v/>
       </c>
       <c r="X12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",D12=""),"",IF(COUNT(D$8:D$13)&lt;2,1,(COUNT(D$8:D$13)-RANK(D12,D$8:D$13,0))/(COUNT(D$8:D$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",D12=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D12,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
         <v/>
       </c>
       <c r="Y12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",E12=""),"",IF(COUNT(E$8:E$13)&lt;2,1,(COUNT(E$8:E$13)-RANK(E12,E$8:E$13,1))/(COUNT(E$8:E$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",E12=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E12,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
         <v/>
       </c>
       <c r="Z12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",F12=""),"",IF(COUNT(F$8:F$13)&lt;2,1,(COUNT(F$8:F$13)-RANK(F12,F$8:F$13,0))/(COUNT(F$8:F$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",F12=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F12,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
         <v/>
       </c>
       <c r="AA12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",G12=""),"",IF(COUNT(G$8:G$13)&lt;2,1,(COUNT(G$8:G$13)-RANK(G12,G$8:G$13,0))/(COUNT(G$8:G$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",G12=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G12,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
         <v/>
       </c>
       <c r="AB12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",J12=""),"",IF(COUNT(J$8:J$13)&lt;2,1,(COUNT(J$8:J$13)-RANK(J12,J$8:J$13,1))/(COUNT(J$8:J$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",J12=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J12,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
         <v/>
       </c>
       <c r="AC12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",P12=""),"",IF(COUNT(P$8:P$13)&lt;2,1,(COUNT(P$8:P$13)-RANK(P12,P$8:P$13,1))/(COUNT(P$8:P$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",P12=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P12,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
         <v/>
       </c>
       <c r="AD12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",S12=""),"",IF(COUNT(S$8:S$13)&lt;2,1,(COUNT(S$8:S$13)-RANK(S12,S$8:S$13,1))/(COUNT(S$8:S$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",S12=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S12,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
         <v/>
       </c>
       <c r="AE12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",T12=""),"",IF(COUNT(T$8:T$13)&lt;2,1,(COUNT(T$8:T$13)-RANK(T12,T$8:T$13,0))/(COUNT(T$8:T$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",T12=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T12,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
         <v/>
       </c>
       <c r="AF12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",U12=""),"",IF(COUNT(U$8:U$13)&lt;2,1,(COUNT(U$8:U$13)-RANK(U12,U$8:U$13,0))/(COUNT(U$8:U$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",U12=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U12,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
         <v/>
       </c>
       <c r="AG12" s="29" t="str">
-        <f aca="false">IF(OR($A12="",V12=""),"",IF(COUNT(V$8:V$13)&lt;2,1,(COUNT(V$8:V$13)-RANK(V12,V$8:V$13,0))/(COUNT(V$8:V$13)-1)))</f>
+        <f aca="false">IF(OR($A12="",V12=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V12,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
         <v/>
       </c>
     </row>
@@ -12316,228 +12316,600 @@
         <v/>
       </c>
       <c r="X13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",D13=""),"",IF(COUNT(D$8:D$13)&lt;2,1,(COUNT(D$8:D$13)-RANK(D13,D$8:D$13,0))/(COUNT(D$8:D$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",D13=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D13,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
         <v/>
       </c>
       <c r="Y13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",E13=""),"",IF(COUNT(E$8:E$13)&lt;2,1,(COUNT(E$8:E$13)-RANK(E13,E$8:E$13,1))/(COUNT(E$8:E$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",E13=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E13,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
         <v/>
       </c>
       <c r="Z13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",F13=""),"",IF(COUNT(F$8:F$13)&lt;2,1,(COUNT(F$8:F$13)-RANK(F13,F$8:F$13,0))/(COUNT(F$8:F$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",F13=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F13,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
         <v/>
       </c>
       <c r="AA13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",G13=""),"",IF(COUNT(G$8:G$13)&lt;2,1,(COUNT(G$8:G$13)-RANK(G13,G$8:G$13,0))/(COUNT(G$8:G$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",G13=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G13,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
         <v/>
       </c>
       <c r="AB13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",J13=""),"",IF(COUNT(J$8:J$13)&lt;2,1,(COUNT(J$8:J$13)-RANK(J13,J$8:J$13,1))/(COUNT(J$8:J$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",J13=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J13,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
         <v/>
       </c>
       <c r="AC13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",P13=""),"",IF(COUNT(P$8:P$13)&lt;2,1,(COUNT(P$8:P$13)-RANK(P13,P$8:P$13,1))/(COUNT(P$8:P$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",P13=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P13,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
         <v/>
       </c>
       <c r="AD13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",S13=""),"",IF(COUNT(S$8:S$13)&lt;2,1,(COUNT(S$8:S$13)-RANK(S13,S$8:S$13,1))/(COUNT(S$8:S$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",S13=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S13,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
         <v/>
       </c>
       <c r="AE13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",T13=""),"",IF(COUNT(T$8:T$13)&lt;2,1,(COUNT(T$8:T$13)-RANK(T13,T$8:T$13,0))/(COUNT(T$8:T$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",T13=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T13,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
         <v/>
       </c>
       <c r="AF13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",U13=""),"",IF(COUNT(U$8:U$13)&lt;2,1,(COUNT(U$8:U$13)-RANK(U13,U$8:U$13,0))/(COUNT(U$8:U$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",U13=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U13,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
         <v/>
       </c>
       <c r="AG13" s="29" t="str">
-        <f aca="false">IF(OR($A13="",V13=""),"",IF(COUNT(V$8:V$13)&lt;2,1,(COUNT(V$8:V$13)-RANK(V13,V$8:V$13,0))/(COUNT(V$8:V$13)-1)))</f>
+        <f aca="false">IF(OR($A13="",V13=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V13,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30"/>
+      <c r="B14" s="21" t="str">
+        <f aca="false">IF($A14="","",COUNTIF(ZIPs!$A$8:$A$107,$A14))</f>
+        <v/>
+      </c>
+      <c r="C14" s="22" t="str">
+        <f aca="false">IF($A14="","",IF($B14=0,"",IFERROR(AVERAGEIFS(ZIPs!$D$8:$D$107,ZIPs!$A$8:$A$107,$A14),"")))</f>
+        <v/>
+      </c>
+      <c r="D14" s="21" t="str">
+        <f aca="false">IF($A14="","",IF($B14=0,"",SUMIFS(ZIPs!$E$8:$E$107,ZIPs!$A$8:$A$107,$A14)))</f>
+        <v/>
+      </c>
+      <c r="E14" s="21" t="str">
+        <f aca="false">IF($A14="","",IF($B14=0,"",IFERROR(AVERAGEIFS(ZIPs!$G$8:$G$107,ZIPs!$A$8:$A$107,$A14),"")))</f>
+        <v/>
+      </c>
+      <c r="F14" s="23" t="str">
+        <f aca="false">IF($A14="","",IF($B14=0,"",IFERROR(AVERAGEIFS(ZIPs!$J$8:$J$107,ZIPs!$A$8:$A$107,$A14),"")))</f>
+        <v/>
+      </c>
+      <c r="G14" s="23" t="str">
+        <f aca="false">IF($A14="","",IF($B14=0,"",IFERROR(AVERAGEIFS(ZIPs!$S$8:$S$107,ZIPs!$A$8:$A$107,$A14),"")))</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="str">
+        <f aca="false">IF($A14="","",IF($B14=0,"",IFERROR(AVERAGEIFS(ZIPs!$T$8:$T$107,ZIPs!$A$8:$A$107,$A14),"")))</f>
+        <v/>
+      </c>
+      <c r="I14" s="21" t="str">
+        <f aca="false">IF($A14="","",COUNTIF('Past Flips'!$A$8:$A$307,$A14)+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A14,'Flip Candidates'!$O$8:$O$207,"Likely flip"))</f>
+        <v/>
+      </c>
+      <c r="J14" s="24" t="str">
+        <f aca="false">IF(OR($A14="",D14="",D14=0),"",I14/(D14*4))</f>
+        <v/>
+      </c>
+      <c r="K14" s="23" t="str">
+        <f aca="false">IF($A14="","",IFERROR((SUMIFS('Past Flips'!$T$8:$T$307,'Past Flips'!$A$8:$A$307,$A14)+SUMIFS('Flip Candidates'!$R$8:$R$207,'Flip Candidates'!$A$8:$A$207,$A14,'Flip Candidates'!$O$8:$O$207,"Likely flip"))/(COUNTIFS('Past Flips'!$A$8:$A$307,$A14,'Past Flips'!$T$8:$T$307,"&lt;&gt;")+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A14,'Flip Candidates'!$O$8:$O$207,"Likely flip")),""))</f>
+        <v/>
+      </c>
+      <c r="L14" s="21" t="str">
+        <f aca="false">IF($A14="","",COUNTIF('Listing Watch'!$A$8:$A$307,$A14))</f>
+        <v/>
+      </c>
+      <c r="M14" s="21" t="str">
+        <f aca="false">IF($A14="","",IFERROR(AVERAGEIFS('Listing Watch'!$S$8:$S$307,'Listing Watch'!$A$8:$A$307,$A14),""))</f>
+        <v/>
+      </c>
+      <c r="N14" s="23" t="str">
+        <f aca="false">IF(OR($A14="",L14=0),"",COUNTIFS('Listing Watch'!$A$8:$A$307,$A14,'Listing Watch'!$R$8:$R$307,"&gt;0")/L14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="21" t="str">
+        <f aca="false">IF($A14="","",COUNTIF(Calls!$A$8:$A$307,$A14))</f>
+        <v/>
+      </c>
+      <c r="P14" s="25" t="str">
+        <f aca="false">IF($A14="","",IFERROR(AVERAGEIFS(Calls!$K$8:$K$307,Calls!$A$8:$A$307,$A14),""))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="22" t="str">
+        <f aca="false">IF($A14="","",IFERROR(AVERAGEIFS(Calls!$G$8:$G$307,Calls!$A$8:$A$307,$A14),""))</f>
+        <v/>
+      </c>
+      <c r="R14" s="22" t="str">
+        <f aca="false">IF($A14="","",IFERROR(AVERAGEIFS(Calls!$H$8:$H$307,Calls!$A$8:$A$307,$A14),""))</f>
+        <v/>
+      </c>
+      <c r="S14" s="21" t="str">
+        <f aca="false">IF($A14="","",IF(COUNTIF(Competition!$A$8:$A$207,$A14)=0,"",COUNTIF(Competition!$A$8:$A$207,$A14)))</f>
+        <v/>
+      </c>
+      <c r="T14" s="31"/>
+      <c r="U14" s="31"/>
+      <c r="V14" s="27"/>
+      <c r="W14" s="28" t="str">
+        <f aca="false">IF($A14="","",IFERROR(ROUND(100*SUMPRODUCT($X$6:$AG$6,X14:AG14)/SUMPRODUCT($X$6:$AG$6,--(X14:AG14&lt;&gt;"")),0),""))</f>
+        <v/>
+      </c>
+      <c r="X14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",D14=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D14,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Y14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",E14=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E14,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Z14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",F14=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F14,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AA14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",G14=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G14,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AB14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",J14=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J14,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AC14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",P14=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P14,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AD14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",S14=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S14,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AE14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",T14=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T14,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AF14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",U14=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U14,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AG14" s="29" t="str">
+        <f aca="false">IF(OR($A14="",V14=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V14,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30"/>
+      <c r="B15" s="21" t="str">
+        <f aca="false">IF($A15="","",COUNTIF(ZIPs!$A$8:$A$107,$A15))</f>
+        <v/>
+      </c>
+      <c r="C15" s="22" t="str">
+        <f aca="false">IF($A15="","",IF($B15=0,"",IFERROR(AVERAGEIFS(ZIPs!$D$8:$D$107,ZIPs!$A$8:$A$107,$A15),"")))</f>
+        <v/>
+      </c>
+      <c r="D15" s="21" t="str">
+        <f aca="false">IF($A15="","",IF($B15=0,"",SUMIFS(ZIPs!$E$8:$E$107,ZIPs!$A$8:$A$107,$A15)))</f>
+        <v/>
+      </c>
+      <c r="E15" s="21" t="str">
+        <f aca="false">IF($A15="","",IF($B15=0,"",IFERROR(AVERAGEIFS(ZIPs!$G$8:$G$107,ZIPs!$A$8:$A$107,$A15),"")))</f>
+        <v/>
+      </c>
+      <c r="F15" s="23" t="str">
+        <f aca="false">IF($A15="","",IF($B15=0,"",IFERROR(AVERAGEIFS(ZIPs!$J$8:$J$107,ZIPs!$A$8:$A$107,$A15),"")))</f>
+        <v/>
+      </c>
+      <c r="G15" s="23" t="str">
+        <f aca="false">IF($A15="","",IF($B15=0,"",IFERROR(AVERAGEIFS(ZIPs!$S$8:$S$107,ZIPs!$A$8:$A$107,$A15),"")))</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="str">
+        <f aca="false">IF($A15="","",IF($B15=0,"",IFERROR(AVERAGEIFS(ZIPs!$T$8:$T$107,ZIPs!$A$8:$A$107,$A15),"")))</f>
+        <v/>
+      </c>
+      <c r="I15" s="21" t="str">
+        <f aca="false">IF($A15="","",COUNTIF('Past Flips'!$A$8:$A$307,$A15)+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A15,'Flip Candidates'!$O$8:$O$207,"Likely flip"))</f>
+        <v/>
+      </c>
+      <c r="J15" s="24" t="str">
+        <f aca="false">IF(OR($A15="",D15="",D15=0),"",I15/(D15*4))</f>
+        <v/>
+      </c>
+      <c r="K15" s="23" t="str">
+        <f aca="false">IF($A15="","",IFERROR((SUMIFS('Past Flips'!$T$8:$T$307,'Past Flips'!$A$8:$A$307,$A15)+SUMIFS('Flip Candidates'!$R$8:$R$207,'Flip Candidates'!$A$8:$A$207,$A15,'Flip Candidates'!$O$8:$O$207,"Likely flip"))/(COUNTIFS('Past Flips'!$A$8:$A$307,$A15,'Past Flips'!$T$8:$T$307,"&lt;&gt;")+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A15,'Flip Candidates'!$O$8:$O$207,"Likely flip")),""))</f>
+        <v/>
+      </c>
+      <c r="L15" s="21" t="str">
+        <f aca="false">IF($A15="","",COUNTIF('Listing Watch'!$A$8:$A$307,$A15))</f>
+        <v/>
+      </c>
+      <c r="M15" s="21" t="str">
+        <f aca="false">IF($A15="","",IFERROR(AVERAGEIFS('Listing Watch'!$S$8:$S$307,'Listing Watch'!$A$8:$A$307,$A15),""))</f>
+        <v/>
+      </c>
+      <c r="N15" s="23" t="str">
+        <f aca="false">IF(OR($A15="",L15=0),"",COUNTIFS('Listing Watch'!$A$8:$A$307,$A15,'Listing Watch'!$R$8:$R$307,"&gt;0")/L15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="21" t="str">
+        <f aca="false">IF($A15="","",COUNTIF(Calls!$A$8:$A$307,$A15))</f>
+        <v/>
+      </c>
+      <c r="P15" s="25" t="str">
+        <f aca="false">IF($A15="","",IFERROR(AVERAGEIFS(Calls!$K$8:$K$307,Calls!$A$8:$A$307,$A15),""))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="22" t="str">
+        <f aca="false">IF($A15="","",IFERROR(AVERAGEIFS(Calls!$G$8:$G$307,Calls!$A$8:$A$307,$A15),""))</f>
+        <v/>
+      </c>
+      <c r="R15" s="22" t="str">
+        <f aca="false">IF($A15="","",IFERROR(AVERAGEIFS(Calls!$H$8:$H$307,Calls!$A$8:$A$307,$A15),""))</f>
+        <v/>
+      </c>
+      <c r="S15" s="21" t="str">
+        <f aca="false">IF($A15="","",IF(COUNTIF(Competition!$A$8:$A$207,$A15)=0,"",COUNTIF(Competition!$A$8:$A$207,$A15)))</f>
+        <v/>
+      </c>
+      <c r="T15" s="31"/>
+      <c r="U15" s="31"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="28" t="str">
+        <f aca="false">IF($A15="","",IFERROR(ROUND(100*SUMPRODUCT($X$6:$AG$6,X15:AG15)/SUMPRODUCT($X$6:$AG$6,--(X15:AG15&lt;&gt;"")),0),""))</f>
+        <v/>
+      </c>
+      <c r="X15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",D15=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D15,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Y15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",E15=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E15,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Z15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",F15=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F15,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AA15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",G15=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G15,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AB15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",J15=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J15,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AC15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",P15=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P15,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AD15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",S15=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S15,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AE15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",T15=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T15,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AF15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",U15=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U15,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AG15" s="29" t="str">
+        <f aca="false">IF(OR($A15="",V15=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V15,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="30"/>
+      <c r="B16" s="21" t="str">
+        <f aca="false">IF($A16="","",COUNTIF(ZIPs!$A$8:$A$107,$A16))</f>
+        <v/>
+      </c>
+      <c r="C16" s="22" t="str">
+        <f aca="false">IF($A16="","",IF($B16=0,"",IFERROR(AVERAGEIFS(ZIPs!$D$8:$D$107,ZIPs!$A$8:$A$107,$A16),"")))</f>
+        <v/>
+      </c>
+      <c r="D16" s="21" t="str">
+        <f aca="false">IF($A16="","",IF($B16=0,"",SUMIFS(ZIPs!$E$8:$E$107,ZIPs!$A$8:$A$107,$A16)))</f>
+        <v/>
+      </c>
+      <c r="E16" s="21" t="str">
+        <f aca="false">IF($A16="","",IF($B16=0,"",IFERROR(AVERAGEIFS(ZIPs!$G$8:$G$107,ZIPs!$A$8:$A$107,$A16),"")))</f>
+        <v/>
+      </c>
+      <c r="F16" s="23" t="str">
+        <f aca="false">IF($A16="","",IF($B16=0,"",IFERROR(AVERAGEIFS(ZIPs!$J$8:$J$107,ZIPs!$A$8:$A$107,$A16),"")))</f>
+        <v/>
+      </c>
+      <c r="G16" s="23" t="str">
+        <f aca="false">IF($A16="","",IF($B16=0,"",IFERROR(AVERAGEIFS(ZIPs!$S$8:$S$107,ZIPs!$A$8:$A$107,$A16),"")))</f>
+        <v/>
+      </c>
+      <c r="H16" s="23" t="str">
+        <f aca="false">IF($A16="","",IF($B16=0,"",IFERROR(AVERAGEIFS(ZIPs!$T$8:$T$107,ZIPs!$A$8:$A$107,$A16),"")))</f>
+        <v/>
+      </c>
+      <c r="I16" s="21" t="str">
+        <f aca="false">IF($A16="","",COUNTIF('Past Flips'!$A$8:$A$307,$A16)+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A16,'Flip Candidates'!$O$8:$O$207,"Likely flip"))</f>
+        <v/>
+      </c>
+      <c r="J16" s="24" t="str">
+        <f aca="false">IF(OR($A16="",D16="",D16=0),"",I16/(D16*4))</f>
+        <v/>
+      </c>
+      <c r="K16" s="23" t="str">
+        <f aca="false">IF($A16="","",IFERROR((SUMIFS('Past Flips'!$T$8:$T$307,'Past Flips'!$A$8:$A$307,$A16)+SUMIFS('Flip Candidates'!$R$8:$R$207,'Flip Candidates'!$A$8:$A$207,$A16,'Flip Candidates'!$O$8:$O$207,"Likely flip"))/(COUNTIFS('Past Flips'!$A$8:$A$307,$A16,'Past Flips'!$T$8:$T$307,"&lt;&gt;")+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A16,'Flip Candidates'!$O$8:$O$207,"Likely flip")),""))</f>
+        <v/>
+      </c>
+      <c r="L16" s="21" t="str">
+        <f aca="false">IF($A16="","",COUNTIF('Listing Watch'!$A$8:$A$307,$A16))</f>
+        <v/>
+      </c>
+      <c r="M16" s="21" t="str">
+        <f aca="false">IF($A16="","",IFERROR(AVERAGEIFS('Listing Watch'!$S$8:$S$307,'Listing Watch'!$A$8:$A$307,$A16),""))</f>
+        <v/>
+      </c>
+      <c r="N16" s="23" t="str">
+        <f aca="false">IF(OR($A16="",L16=0),"",COUNTIFS('Listing Watch'!$A$8:$A$307,$A16,'Listing Watch'!$R$8:$R$307,"&gt;0")/L16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="21" t="str">
+        <f aca="false">IF($A16="","",COUNTIF(Calls!$A$8:$A$307,$A16))</f>
+        <v/>
+      </c>
+      <c r="P16" s="25" t="str">
+        <f aca="false">IF($A16="","",IFERROR(AVERAGEIFS(Calls!$K$8:$K$307,Calls!$A$8:$A$307,$A16),""))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="22" t="str">
+        <f aca="false">IF($A16="","",IFERROR(AVERAGEIFS(Calls!$G$8:$G$307,Calls!$A$8:$A$307,$A16),""))</f>
+        <v/>
+      </c>
+      <c r="R16" s="22" t="str">
+        <f aca="false">IF($A16="","",IFERROR(AVERAGEIFS(Calls!$H$8:$H$307,Calls!$A$8:$A$307,$A16),""))</f>
+        <v/>
+      </c>
+      <c r="S16" s="21" t="str">
+        <f aca="false">IF($A16="","",IF(COUNTIF(Competition!$A$8:$A$207,$A16)=0,"",COUNTIF(Competition!$A$8:$A$207,$A16)))</f>
+        <v/>
+      </c>
+      <c r="T16" s="31"/>
+      <c r="U16" s="31"/>
+      <c r="V16" s="27"/>
+      <c r="W16" s="28" t="str">
+        <f aca="false">IF($A16="","",IFERROR(ROUND(100*SUMPRODUCT($X$6:$AG$6,X16:AG16)/SUMPRODUCT($X$6:$AG$6,--(X16:AG16&lt;&gt;"")),0),""))</f>
+        <v/>
+      </c>
+      <c r="X16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",D16=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D16,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Y16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",E16=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E16,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Z16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",F16=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F16,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AA16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",G16=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G16,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AB16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",J16=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J16,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AC16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",P16=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P16,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AD16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",S16=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S16,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AE16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",T16=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T16,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AF16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",U16=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U16,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AG16" s="29" t="str">
+        <f aca="false">IF(OR($A16="",V16=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V16,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30"/>
+      <c r="B17" s="21" t="str">
+        <f aca="false">IF($A17="","",COUNTIF(ZIPs!$A$8:$A$107,$A17))</f>
+        <v/>
+      </c>
+      <c r="C17" s="22" t="str">
+        <f aca="false">IF($A17="","",IF($B17=0,"",IFERROR(AVERAGEIFS(ZIPs!$D$8:$D$107,ZIPs!$A$8:$A$107,$A17),"")))</f>
+        <v/>
+      </c>
+      <c r="D17" s="21" t="str">
+        <f aca="false">IF($A17="","",IF($B17=0,"",SUMIFS(ZIPs!$E$8:$E$107,ZIPs!$A$8:$A$107,$A17)))</f>
+        <v/>
+      </c>
+      <c r="E17" s="21" t="str">
+        <f aca="false">IF($A17="","",IF($B17=0,"",IFERROR(AVERAGEIFS(ZIPs!$G$8:$G$107,ZIPs!$A$8:$A$107,$A17),"")))</f>
+        <v/>
+      </c>
+      <c r="F17" s="23" t="str">
+        <f aca="false">IF($A17="","",IF($B17=0,"",IFERROR(AVERAGEIFS(ZIPs!$J$8:$J$107,ZIPs!$A$8:$A$107,$A17),"")))</f>
+        <v/>
+      </c>
+      <c r="G17" s="23" t="str">
+        <f aca="false">IF($A17="","",IF($B17=0,"",IFERROR(AVERAGEIFS(ZIPs!$S$8:$S$107,ZIPs!$A$8:$A$107,$A17),"")))</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="str">
+        <f aca="false">IF($A17="","",IF($B17=0,"",IFERROR(AVERAGEIFS(ZIPs!$T$8:$T$107,ZIPs!$A$8:$A$107,$A17),"")))</f>
+        <v/>
+      </c>
+      <c r="I17" s="21" t="str">
+        <f aca="false">IF($A17="","",COUNTIF('Past Flips'!$A$8:$A$307,$A17)+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A17,'Flip Candidates'!$O$8:$O$207,"Likely flip"))</f>
+        <v/>
+      </c>
+      <c r="J17" s="24" t="str">
+        <f aca="false">IF(OR($A17="",D17="",D17=0),"",I17/(D17*4))</f>
+        <v/>
+      </c>
+      <c r="K17" s="23" t="str">
+        <f aca="false">IF($A17="","",IFERROR((SUMIFS('Past Flips'!$T$8:$T$307,'Past Flips'!$A$8:$A$307,$A17)+SUMIFS('Flip Candidates'!$R$8:$R$207,'Flip Candidates'!$A$8:$A$207,$A17,'Flip Candidates'!$O$8:$O$207,"Likely flip"))/(COUNTIFS('Past Flips'!$A$8:$A$307,$A17,'Past Flips'!$T$8:$T$307,"&lt;&gt;")+COUNTIFS('Flip Candidates'!$A$8:$A$207,$A17,'Flip Candidates'!$O$8:$O$207,"Likely flip")),""))</f>
+        <v/>
+      </c>
+      <c r="L17" s="21" t="str">
+        <f aca="false">IF($A17="","",COUNTIF('Listing Watch'!$A$8:$A$307,$A17))</f>
+        <v/>
+      </c>
+      <c r="M17" s="21" t="str">
+        <f aca="false">IF($A17="","",IFERROR(AVERAGEIFS('Listing Watch'!$S$8:$S$307,'Listing Watch'!$A$8:$A$307,$A17),""))</f>
+        <v/>
+      </c>
+      <c r="N17" s="23" t="str">
+        <f aca="false">IF(OR($A17="",L17=0),"",COUNTIFS('Listing Watch'!$A$8:$A$307,$A17,'Listing Watch'!$R$8:$R$307,"&gt;0")/L17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="21" t="str">
+        <f aca="false">IF($A17="","",COUNTIF(Calls!$A$8:$A$307,$A17))</f>
+        <v/>
+      </c>
+      <c r="P17" s="25" t="str">
+        <f aca="false">IF($A17="","",IFERROR(AVERAGEIFS(Calls!$K$8:$K$307,Calls!$A$8:$A$307,$A17),""))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="22" t="str">
+        <f aca="false">IF($A17="","",IFERROR(AVERAGEIFS(Calls!$G$8:$G$307,Calls!$A$8:$A$307,$A17),""))</f>
+        <v/>
+      </c>
+      <c r="R17" s="22" t="str">
+        <f aca="false">IF($A17="","",IFERROR(AVERAGEIFS(Calls!$H$8:$H$307,Calls!$A$8:$A$307,$A17),""))</f>
+        <v/>
+      </c>
+      <c r="S17" s="21" t="str">
+        <f aca="false">IF($A17="","",IF(COUNTIF(Competition!$A$8:$A$207,$A17)=0,"",COUNTIF(Competition!$A$8:$A$207,$A17)))</f>
+        <v/>
+      </c>
+      <c r="T17" s="31"/>
+      <c r="U17" s="31"/>
+      <c r="V17" s="27"/>
+      <c r="W17" s="28" t="str">
+        <f aca="false">IF($A17="","",IFERROR(ROUND(100*SUMPRODUCT($X$6:$AG$6,X17:AG17)/SUMPRODUCT($X$6:$AG$6,--(X17:AG17&lt;&gt;"")),0),""))</f>
+        <v/>
+      </c>
+      <c r="X17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",D17=""),"",IF(COUNT(D$8:D$17)&lt;2,1,(COUNT(D$8:D$17)-RANK(D17,D$8:D$17,0))/(COUNT(D$8:D$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Y17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",E17=""),"",IF(COUNT(E$8:E$17)&lt;2,1,(COUNT(E$8:E$17)-RANK(E17,E$8:E$17,1))/(COUNT(E$8:E$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="Z17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",F17=""),"",IF(COUNT(F$8:F$17)&lt;2,1,(COUNT(F$8:F$17)-RANK(F17,F$8:F$17,0))/(COUNT(F$8:F$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AA17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",G17=""),"",IF(COUNT(G$8:G$17)&lt;2,1,(COUNT(G$8:G$17)-RANK(G17,G$8:G$17,0))/(COUNT(G$8:G$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AB17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",J17=""),"",IF(COUNT(J$8:J$17)&lt;2,1,(COUNT(J$8:J$17)-RANK(J17,J$8:J$17,1))/(COUNT(J$8:J$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AC17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",P17=""),"",IF(COUNT(P$8:P$17)&lt;2,1,(COUNT(P$8:P$17)-RANK(P17,P$8:P$17,1))/(COUNT(P$8:P$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AD17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",S17=""),"",IF(COUNT(S$8:S$17)&lt;2,1,(COUNT(S$8:S$17)-RANK(S17,S$8:S$17,1))/(COUNT(S$8:S$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AE17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",T17=""),"",IF(COUNT(T$8:T$17)&lt;2,1,(COUNT(T$8:T$17)-RANK(T17,T$8:T$17,0))/(COUNT(T$8:T$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AF17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",U17=""),"",IF(COUNT(U$8:U$17)&lt;2,1,(COUNT(U$8:U$17)-RANK(U17,U$8:U$17,0))/(COUNT(U$8:U$17)-1)))</f>
+        <v/>
+      </c>
+      <c r="AG17" s="29" t="str">
+        <f aca="false">IF(OR($A17="",V17=""),"",IF(COUNT(V$8:V$17)&lt;2,1,(COUNT(V$8:V$17)-RANK(V17,V$8:V$17,0))/(COUNT(V$8:V$17)-1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+    <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B21" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C21" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D21" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E21" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F21" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G21" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H21" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="I21" s="19" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="str">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="str">
         <f aca="false">IF($A$8="","",$A$8)</f>
         <v>Sampleville, OH</v>
-      </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="33" t="str">
-        <f aca="false">IF($A18="","",IF(COUNTIF(Calls!$A$8:$A$307,$A18)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A18)&amp;"/10)"))</f>
-        <v>No (1/10)</v>
-      </c>
-      <c r="D18" s="33" t="str">
-        <f aca="false">IF($A18="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A18,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A18,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
-        <v>No (1/3)</v>
-      </c>
-      <c r="E18" s="32"/>
-      <c r="F18" s="33" t="str">
-        <f aca="false">IF($A18="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A18)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A18)&amp;"/10)"))</f>
-        <v>No (1/10)</v>
-      </c>
-      <c r="G18" s="33" t="str">
-        <f aca="false">IF($A18="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A18,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A18)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A18),"0%")&amp;")")))</f>
-        <v>Yes</v>
-      </c>
-      <c r="H18" s="32"/>
-      <c r="I18" s="34" t="str">
-        <f aca="false">IF($A18="","",IF(AND(UPPER(B18)="Y",C18="Yes",D18="Yes",UPPER(E18)="Y",F18="Yes",G18="Yes",UPPER(H18)="Y"),"READY","Not yet"))</f>
-        <v>Not yet</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="str">
-        <f aca="false">IF($A$9="","",$A$9)</f>
-        <v/>
-      </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="33" t="str">
-        <f aca="false">IF($A19="","",IF(COUNTIF(Calls!$A$8:$A$307,$A19)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A19)&amp;"/10)"))</f>
-        <v/>
-      </c>
-      <c r="D19" s="33" t="str">
-        <f aca="false">IF($A19="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A19,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A19,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
-        <v/>
-      </c>
-      <c r="E19" s="32"/>
-      <c r="F19" s="33" t="str">
-        <f aca="false">IF($A19="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A19)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A19)&amp;"/10)"))</f>
-        <v/>
-      </c>
-      <c r="G19" s="33" t="str">
-        <f aca="false">IF($A19="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A19,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A19)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A19),"0%")&amp;")")))</f>
-        <v/>
-      </c>
-      <c r="H19" s="32"/>
-      <c r="I19" s="34" t="str">
-        <f aca="false">IF($A19="","",IF(AND(UPPER(B19)="Y",C19="Yes",D19="Yes",UPPER(E19)="Y",F19="Yes",G19="Yes",UPPER(H19)="Y"),"READY","Not yet"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="str">
-        <f aca="false">IF($A$10="","",$A$10)</f>
-        <v/>
-      </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="33" t="str">
-        <f aca="false">IF($A20="","",IF(COUNTIF(Calls!$A$8:$A$307,$A20)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A20)&amp;"/10)"))</f>
-        <v/>
-      </c>
-      <c r="D20" s="33" t="str">
-        <f aca="false">IF($A20="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A20,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A20,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
-        <v/>
-      </c>
-      <c r="E20" s="32"/>
-      <c r="F20" s="33" t="str">
-        <f aca="false">IF($A20="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A20)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A20)&amp;"/10)"))</f>
-        <v/>
-      </c>
-      <c r="G20" s="33" t="str">
-        <f aca="false">IF($A20="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A20,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A20)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A20),"0%")&amp;")")))</f>
-        <v/>
-      </c>
-      <c r="H20" s="32"/>
-      <c r="I20" s="34" t="str">
-        <f aca="false">IF($A20="","",IF(AND(UPPER(B20)="Y",C20="Yes",D20="Yes",UPPER(E20)="Y",F20="Yes",G20="Yes",UPPER(H20)="Y"),"READY","Not yet"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="str">
-        <f aca="false">IF($A$11="","",$A$11)</f>
-        <v/>
-      </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="33" t="str">
-        <f aca="false">IF($A21="","",IF(COUNTIF(Calls!$A$8:$A$307,$A21)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A21)&amp;"/10)"))</f>
-        <v/>
-      </c>
-      <c r="D21" s="33" t="str">
-        <f aca="false">IF($A21="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A21,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A21,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
-        <v/>
-      </c>
-      <c r="E21" s="32"/>
-      <c r="F21" s="33" t="str">
-        <f aca="false">IF($A21="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A21)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A21)&amp;"/10)"))</f>
-        <v/>
-      </c>
-      <c r="G21" s="33" t="str">
-        <f aca="false">IF($A21="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A21,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A21)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A21),"0%")&amp;")")))</f>
-        <v/>
-      </c>
-      <c r="H21" s="32"/>
-      <c r="I21" s="34" t="str">
-        <f aca="false">IF($A21="","",IF(AND(UPPER(B21)="Y",C21="Yes",D21="Yes",UPPER(E21)="Y",F21="Yes",G21="Yes",UPPER(H21)="Y"),"READY","Not yet"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="str">
-        <f aca="false">IF($A$12="","",$A$12)</f>
-        <v/>
       </c>
       <c r="B22" s="32"/>
       <c r="C22" s="33" t="str">
         <f aca="false">IF($A22="","",IF(COUNTIF(Calls!$A$8:$A$307,$A22)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A22)&amp;"/10)"))</f>
-        <v/>
+        <v>No (1/10)</v>
       </c>
       <c r="D22" s="33" t="str">
         <f aca="false">IF($A22="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A22,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A22,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
-        <v/>
+        <v>No (1/3)</v>
       </c>
       <c r="E22" s="32"/>
       <c r="F22" s="33" t="str">
         <f aca="false">IF($A22="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A22)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A22)&amp;"/10)"))</f>
-        <v/>
+        <v>No (1/10)</v>
       </c>
       <c r="G22" s="33" t="str">
         <f aca="false">IF($A22="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A22,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A22)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A22),"0%")&amp;")")))</f>
-        <v/>
+        <v>Yes</v>
       </c>
       <c r="H22" s="32"/>
       <c r="I22" s="34" t="str">
         <f aca="false">IF($A22="","",IF(AND(UPPER(B22)="Y",C22="Yes",D22="Yes",UPPER(E22)="Y",F22="Yes",G22="Yes",UPPER(H22)="Y"),"READY","Not yet"))</f>
-        <v/>
+        <v>Not yet</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="str">
-        <f aca="false">IF($A$13="","",$A$13)</f>
+        <f aca="false">IF($A$9="","",$A$9)</f>
         <v/>
       </c>
       <c r="B23" s="32"/>
@@ -12564,8 +12936,240 @@
         <v/>
       </c>
     </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="str">
+        <f aca="false">IF($A$10="","",$A$10)</f>
+        <v/>
+      </c>
+      <c r="B24" s="32"/>
+      <c r="C24" s="33" t="str">
+        <f aca="false">IF($A24="","",IF(COUNTIF(Calls!$A$8:$A$307,$A24)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A24)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D24" s="33" t="str">
+        <f aca="false">IF($A24="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A24,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A24,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E24" s="32"/>
+      <c r="F24" s="33" t="str">
+        <f aca="false">IF($A24="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A24)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A24)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G24" s="33" t="str">
+        <f aca="false">IF($A24="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A24,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A24)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A24),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H24" s="32"/>
+      <c r="I24" s="34" t="str">
+        <f aca="false">IF($A24="","",IF(AND(UPPER(B24)="Y",C24="Yes",D24="Yes",UPPER(E24)="Y",F24="Yes",G24="Yes",UPPER(H24)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="6" t="str">
+        <f aca="false">IF($A$11="","",$A$11)</f>
+        <v/>
+      </c>
+      <c r="B25" s="32"/>
+      <c r="C25" s="33" t="str">
+        <f aca="false">IF($A25="","",IF(COUNTIF(Calls!$A$8:$A$307,$A25)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A25)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D25" s="33" t="str">
+        <f aca="false">IF($A25="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A25,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A25,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E25" s="32"/>
+      <c r="F25" s="33" t="str">
+        <f aca="false">IF($A25="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A25)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A25)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="33" t="str">
+        <f aca="false">IF($A25="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A25,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A25)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A25),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H25" s="32"/>
+      <c r="I25" s="34" t="str">
+        <f aca="false">IF($A25="","",IF(AND(UPPER(B25)="Y",C25="Yes",D25="Yes",UPPER(E25)="Y",F25="Yes",G25="Yes",UPPER(H25)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="str">
+        <f aca="false">IF($A$12="","",$A$12)</f>
+        <v/>
+      </c>
+      <c r="B26" s="32"/>
+      <c r="C26" s="33" t="str">
+        <f aca="false">IF($A26="","",IF(COUNTIF(Calls!$A$8:$A$307,$A26)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A26)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D26" s="33" t="str">
+        <f aca="false">IF($A26="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A26,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A26,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E26" s="32"/>
+      <c r="F26" s="33" t="str">
+        <f aca="false">IF($A26="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A26)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A26)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G26" s="33" t="str">
+        <f aca="false">IF($A26="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A26,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A26)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A26),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H26" s="32"/>
+      <c r="I26" s="34" t="str">
+        <f aca="false">IF($A26="","",IF(AND(UPPER(B26)="Y",C26="Yes",D26="Yes",UPPER(E26)="Y",F26="Yes",G26="Yes",UPPER(H26)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="str">
+        <f aca="false">IF($A$13="","",$A$13)</f>
+        <v/>
+      </c>
+      <c r="B27" s="32"/>
+      <c r="C27" s="33" t="str">
+        <f aca="false">IF($A27="","",IF(COUNTIF(Calls!$A$8:$A$307,$A27)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A27)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D27" s="33" t="str">
+        <f aca="false">IF($A27="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A27,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A27,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E27" s="32"/>
+      <c r="F27" s="33" t="str">
+        <f aca="false">IF($A27="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A27)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A27)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G27" s="33" t="str">
+        <f aca="false">IF($A27="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A27,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A27)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A27),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H27" s="32"/>
+      <c r="I27" s="34" t="str">
+        <f aca="false">IF($A27="","",IF(AND(UPPER(B27)="Y",C27="Yes",D27="Yes",UPPER(E27)="Y",F27="Yes",G27="Yes",UPPER(H27)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="str">
+        <f aca="false">IF($A$14="","",$A$14)</f>
+        <v/>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="33" t="str">
+        <f aca="false">IF($A28="","",IF(COUNTIF(Calls!$A$8:$A$307,$A28)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A28)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D28" s="33" t="str">
+        <f aca="false">IF($A28="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A28,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A28,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E28" s="32"/>
+      <c r="F28" s="33" t="str">
+        <f aca="false">IF($A28="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A28)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A28)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G28" s="33" t="str">
+        <f aca="false">IF($A28="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A28,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A28)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A28),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H28" s="32"/>
+      <c r="I28" s="34" t="str">
+        <f aca="false">IF($A28="","",IF(AND(UPPER(B28)="Y",C28="Yes",D28="Yes",UPPER(E28)="Y",F28="Yes",G28="Yes",UPPER(H28)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="str">
+        <f aca="false">IF($A$15="","",$A$15)</f>
+        <v/>
+      </c>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33" t="str">
+        <f aca="false">IF($A29="","",IF(COUNTIF(Calls!$A$8:$A$307,$A29)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A29)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D29" s="33" t="str">
+        <f aca="false">IF($A29="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A29,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A29,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E29" s="32"/>
+      <c r="F29" s="33" t="str">
+        <f aca="false">IF($A29="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A29)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A29)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G29" s="33" t="str">
+        <f aca="false">IF($A29="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A29,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A29)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A29),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H29" s="32"/>
+      <c r="I29" s="34" t="str">
+        <f aca="false">IF($A29="","",IF(AND(UPPER(B29)="Y",C29="Yes",D29="Yes",UPPER(E29)="Y",F29="Yes",G29="Yes",UPPER(H29)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="str">
+        <f aca="false">IF($A$16="","",$A$16)</f>
+        <v/>
+      </c>
+      <c r="B30" s="32"/>
+      <c r="C30" s="33" t="str">
+        <f aca="false">IF($A30="","",IF(COUNTIF(Calls!$A$8:$A$307,$A30)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A30)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D30" s="33" t="str">
+        <f aca="false">IF($A30="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A30,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A30,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E30" s="32"/>
+      <c r="F30" s="33" t="str">
+        <f aca="false">IF($A30="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A30)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A30)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G30" s="33" t="str">
+        <f aca="false">IF($A30="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A30,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A30)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A30),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H30" s="32"/>
+      <c r="I30" s="34" t="str">
+        <f aca="false">IF($A30="","",IF(AND(UPPER(B30)="Y",C30="Yes",D30="Yes",UPPER(E30)="Y",F30="Yes",G30="Yes",UPPER(H30)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="str">
+        <f aca="false">IF($A$17="","",$A$17)</f>
+        <v/>
+      </c>
+      <c r="B31" s="32"/>
+      <c r="C31" s="33" t="str">
+        <f aca="false">IF($A31="","",IF(COUNTIF(Calls!$A$8:$A$307,$A31)&gt;=10,"Yes","No ("&amp;COUNTIF(Calls!$A$8:$A$307,$A31)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="D31" s="33" t="str">
+        <f aca="false">IF($A31="","",IF(COUNTIFS(Calls!$A$8:$A$307,$A31,Calls!$D$8:$D$307,"Agent")&gt;=3,"Yes","No ("&amp;COUNTIFS(Calls!$A$8:$A$307,$A31,Calls!$D$8:$D$307,"Agent")&amp;"/3)"))</f>
+        <v/>
+      </c>
+      <c r="E31" s="32"/>
+      <c r="F31" s="33" t="str">
+        <f aca="false">IF($A31="","",IF(COUNTIF('Paper Flips'!$B$8:$B$307,$A31)&gt;=10,"Yes","No ("&amp;COUNTIF('Paper Flips'!$B$8:$B$307,$A31)&amp;"/10)"))</f>
+        <v/>
+      </c>
+      <c r="G31" s="33" t="str">
+        <f aca="false">IF($A31="","",IF(COUNTIFS('Paper Flips'!$B$8:$B$307,$A31,'Paper Flips'!$O$8:$O$307,"&lt;&gt;")=0,"No data yet",IF(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A31)&lt;=0.1,"Yes","No ("&amp;TEXT(AVERAGEIFS('Paper Flips'!$O$8:$O$307,'Paper Flips'!$B$8:$B$307,$A31),"0%")&amp;")")))</f>
+        <v/>
+      </c>
+      <c r="H31" s="32"/>
+      <c r="I31" s="34" t="str">
+        <f aca="false">IF($A31="","",IF(AND(UPPER(B31)="Y",C31="Yes",D31="Yes",UPPER(E31)="Y",F31="Yes",G31="Yes",UPPER(H31)="Y"),"READY","Not yet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
         <v>137</v>
       </c>
     </row>
@@ -12577,7 +13181,7 @@
     <mergeCell ref="O6:R6"/>
     <mergeCell ref="T6:V6"/>
   </mergeCells>
-  <conditionalFormatting sqref="W8:W13">
+  <conditionalFormatting sqref="W8:W17">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -12589,7 +13193,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I18:I23">
+  <conditionalFormatting sqref="I22:I31">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"READY"</formula>
     </cfRule>
@@ -12598,11 +13202,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="V8:V13" type="whole">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="V8:V17" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B18:B23 E18:E23 H18:H23" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B22:B31 E22:E31 H22:H31" type="list">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>